<commit_message>
Normalize workbook metadata and re-render demo caption
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/revenue-analysis.xlsx
+++ b/dist/revenue-analysis.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptive Review" sheetId="1" r:id="R8e0d64fbad9d487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning Sensitivity" sheetId="2" r:id="Rede575f492b547bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Attribution" sheetId="3" r:id="R9ec9c46a130d4c73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Calculation" sheetId="4" r:id="R9abb767da72b4406"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition Reconciliation" sheetId="5" r:id="R61efcf2e0e914da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition Appendix" sheetId="6" r:id="R6d9bc16ead484c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Inputs" sheetId="7" r:id="R86b83919773b41c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptive Review" sheetId="1" r:id="Rc351c020ca0d4c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning Sensitivity" sheetId="2" r:id="Re472cbec86394a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Attribution" sheetId="3" r:id="Re030b73205e745e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Calculation" sheetId="4" r:id="R2c942ea5bd08413c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition Reconciliation" sheetId="5" r:id="R31629eabdac84096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition Appendix" sheetId="6" r:id="R60b75b7a74124a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Inputs" sheetId="7" r:id="R65c49eb3bf9648b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -441,7 +441,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rde58fec230e74d40"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R42d1a15c28df489b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -451,9 +451,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -503,7 +503,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1021,7 +1021,7 @@
     <x:mergeCell ref="C29:N29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d91a155dd844c70"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb63dce2e3e124c96"/>
 </x:worksheet>
 </file>
 

</xml_diff>